<commit_message>
Update team member names: Arpita Singh, Aryan Chaudhary, Jyoti Gupta
</commit_message>
<xml_diff>
--- a/Test_Cases_Execution_Sheet.xlsx
+++ b/Test_Cases_Execution_Sheet.xlsx
@@ -206,7 +206,7 @@
     <t>SearchSortTest.java</t>
   </si>
   <si>
-    <t>Teammate 2</t>
+    <t>Arpita Singh</t>
   </si>
   <si>
     <t>search-testing</t>
@@ -236,7 +236,7 @@
     <t>CartTest.java</t>
   </si>
   <si>
-    <t>Teammate 3</t>
+    <t>Aryan Chaudhary</t>
   </si>
   <si>
     <t>cart-testing</t>
@@ -266,7 +266,7 @@
     <t>CheckoutTest.java</t>
   </si>
   <si>
-    <t>Teammate 4</t>
+    <t>Jyoti Gupta</t>
   </si>
   <si>
     <t>checkout-testing</t>
@@ -1519,7 +1519,7 @@
     <col min="8" max="8" width="50.7142857142857" style="1" customWidth="1"/>
     <col min="9" max="9" width="20.2857142857143" customWidth="1"/>
     <col min="10" max="10" width="32.2857142857143" customWidth="1"/>
-    <col min="11" max="11" width="12.7142857142857" customWidth="1"/>
+    <col min="11" max="11" width="17.4285714285714" customWidth="1"/>
     <col min="12" max="12" width="17.2857142857143" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
Implement enterprise Maven + TestNG Page Object Model framework for OrangeHRM
</commit_message>
<xml_diff>
--- a/Test_Cases_Execution_Sheet.xlsx
+++ b/Test_Cases_Execution_Sheet.xlsx
@@ -7,7 +7,7 @@
     <workbookView/>
   </bookViews>
   <sheets>
-    <sheet name="Test Execution &amp; Defects" sheetId="1" r:id="rId1"/>
+    <sheet name="OrangeHRM Test Execution" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="74">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -65,229 +65,190 @@
     <t>Git Commit / PR</t>
   </si>
   <si>
-    <t>TC_SMOKE_01</t>
-  </si>
-  <si>
-    <t>Smoke / Sanity</t>
-  </si>
-  <si>
-    <t>Verify WebDriver launch &amp; site connectivity</t>
-  </si>
-  <si>
-    <t>https://example.com</t>
+    <t>TC_LOG_01</t>
+  </si>
+  <si>
+    <t>Login &amp; Auth</t>
+  </si>
+  <si>
+    <t>Verify successful login with valid credentials and session logout</t>
+  </si>
+  <si>
+    <t>Admin / admin123</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>DEF-001</t>
+  </si>
+  <si>
+    <t>TimeoutException: Timed out waiting for dashboard breadcrumb header after login.</t>
+  </si>
+  <si>
+    <t>OrangeHRM's Vue.js SPA takes a moment to transition URL to /dashboard/index. Fixed by adding wait.until(urlContains('/dashboard')) and dynamic header locator in DashboardPage.</t>
   </si>
   <si>
     <t>PASS</t>
   </si>
   <si>
+    <t>LoginTest.java</t>
+  </si>
+  <si>
+    <t>Manas (Lead)</t>
+  </si>
+  <si>
+    <t>login-testing / PR #1</t>
+  </si>
+  <si>
+    <t>TC_LOG_02</t>
+  </si>
+  <si>
+    <t>Verify login rejection with invalid credentials</t>
+  </si>
+  <si>
+    <t>InvalidUser / WrongPassword123</t>
+  </si>
+  <si>
+    <t>DEF-002</t>
+  </si>
+  <si>
+    <t>AssertionError: Test expected exact text 'Invalid credentials' but alert contained leading icon markup.</t>
+  </si>
+  <si>
+    <t>Locator matched raw container. Fixed by targeting inner text element .oxd-alert-content-text with .contains('Invalid credentials').</t>
+  </si>
+  <si>
+    <t>TC_LOG_03</t>
+  </si>
+  <si>
+    <t>Verify field validation when username is omitted</t>
+  </si>
+  <si>
+    <t>Password: admin123</t>
+  </si>
+  <si>
     <t>None</t>
   </si>
   <si>
-    <t>N/A - Clean run</t>
-  </si>
-  <si>
-    <t>Browser binary and driver matched successfully</t>
-  </si>
-  <si>
-    <t>FirstTest.java</t>
-  </si>
-  <si>
-    <t>Manas</t>
-  </si>
-  <si>
-    <t>f516d27 / PR #1</t>
-  </si>
-  <si>
-    <t>TC_LOG_01</t>
-  </si>
-  <si>
-    <t>Login</t>
-  </si>
-  <si>
-    <t>Verify valid login and user session logout</t>
-  </si>
-  <si>
-    <t>standard_user / secret_sauce</t>
-  </si>
-  <si>
-    <t>FAIL</t>
-  </si>
-  <si>
-    <t>DEF-001</t>
-  </si>
-  <si>
-    <t>TimeoutException: Could not locate login-button after logout. Sidebar animation intercepted click.</t>
-  </si>
-  <si>
-    <t>React burger menu animation delay caused click to be missed. Fixed by using JavascriptExecutor click and explicit WebDriverWait.</t>
-  </si>
-  <si>
-    <t>LoginValidTest.java</t>
-  </si>
-  <si>
-    <t>TC_LOG_02</t>
-  </si>
-  <si>
-    <t>Verify invalid credentials error notification</t>
-  </si>
-  <si>
-    <t>invalid_user / wrong_password</t>
-  </si>
-  <si>
-    <t>DEF-002</t>
-  </si>
-  <si>
-    <t>AssertionError: Test expected exact text 'Invalid credentials' but received 'Epic sadface: Username and password do not match...'.</t>
-  </si>
-  <si>
-    <t>Hardcoded locator text mismatch. Fixed by using flexible substring match (.contains()) and dynamic CSS locator [data-test='error'].</t>
-  </si>
-  <si>
-    <t>LoginInvalidTest.java</t>
-  </si>
-  <si>
-    <t>TC_LOG_03</t>
-  </si>
-  <si>
-    <t>Verify empty credentials field validation</t>
-  </si>
-  <si>
-    <t>Blank fields</t>
-  </si>
-  <si>
     <t>N/A - Clean validation</t>
   </si>
   <si>
-    <t>Both required field validation alerts triggered correctly</t>
-  </si>
-  <si>
-    <t>LoginEmptyCredentialsTest.java</t>
+    <t>Triggered .oxd-input-field-error-message displaying 'Required'</t>
   </si>
   <si>
     <t>TC_LOG_04</t>
   </si>
   <si>
-    <t>Verify account lockout error handling</t>
-  </si>
-  <si>
-    <t>locked_out_user / secret_sauce</t>
-  </si>
-  <si>
-    <t>N/A - Clean lockout validation</t>
-  </si>
-  <si>
-    <t>Lockout alert displayed and verified as expected</t>
-  </si>
-  <si>
-    <t>LoginLockedOutTest.java</t>
-  </si>
-  <si>
-    <t>TC_SRCH_01</t>
-  </si>
-  <si>
-    <t>Catalog / Search</t>
-  </si>
-  <si>
-    <t>Verify sorting products by Price (Low to High)</t>
-  </si>
-  <si>
-    <t>Sort dropdown = 'lohi'</t>
+    <t>Verify field validation when password is omitted</t>
+  </si>
+  <si>
+    <t>Username: Admin</t>
+  </si>
+  <si>
+    <t>TC_LOG_05</t>
+  </si>
+  <si>
+    <t>Verify navigation to Forgot Password recovery page</t>
+  </si>
+  <si>
+    <t>Click 'Forgot your password?'</t>
+  </si>
+  <si>
+    <t>N/A - Clean navigation</t>
+  </si>
+  <si>
+    <t>Navigated to requestPasswordResetCode page successfully</t>
+  </si>
+  <si>
+    <t>TC_ADM_01</t>
+  </si>
+  <si>
+    <t>Admin / Users</t>
+  </si>
+  <si>
+    <t>Verify searching system users by username in Admin module</t>
+  </si>
+  <si>
+    <t>Username = 'Admin'</t>
   </si>
   <si>
     <t>DEF-003</t>
   </si>
   <si>
-    <t>Sorting verification failed: Items sorted alphabetically instead of numerically ($7.99 came after $29.99).</t>
-  </si>
-  <si>
-    <t>Extracted price strings as raw text without stripping '$' and parsing to Double. Fixed parsing logic in assertion.</t>
-  </si>
-  <si>
-    <t>SearchSortTest.java</t>
+    <t>ElementClickInterceptedException: Admin menu item click intercepted by loading spinner overlay.</t>
+  </si>
+  <si>
+    <t>Single-page app initial overlay prevented menu click. Added explicit wait for spinner disappearance before clicking Admin menu.</t>
+  </si>
+  <si>
+    <t>AdminTest.java</t>
   </si>
   <si>
     <t>Arpita Singh</t>
   </si>
   <si>
-    <t>search-testing</t>
-  </si>
-  <si>
-    <t>TC_CART_01</t>
-  </si>
-  <si>
-    <t>Shopping Cart</t>
-  </si>
-  <si>
-    <t>Verify cart badge counter increments on Add to Cart</t>
-  </si>
-  <si>
-    <t>Sauce Labs Backpack</t>
+    <t>admin-testing</t>
+  </si>
+  <si>
+    <t>TC_PIM_01</t>
+  </si>
+  <si>
+    <t>PIM / Employees</t>
+  </si>
+  <si>
+    <t>Verify employee search in PIM employee list</t>
+  </si>
+  <si>
+    <t>Employee Name = 'John'</t>
   </si>
   <si>
     <t>DEF-004</t>
   </si>
   <si>
-    <t>NoSuchElementException: Cart badge element could not be found before item was added.</t>
-  </si>
-  <si>
-    <t>Attempted to assert cart badge visibility when cart was empty (badge element is absent in DOM until first item added). Added condition check.</t>
-  </si>
-  <si>
-    <t>CartTest.java</t>
+    <t>NoSuchElementException: Employee table card element not found in DOM before search completed.</t>
+  </si>
+  <si>
+    <t>AJAX search table loads asynchronously. Replaced implicit delay with explicit wait for .oxd-table-card visibility.</t>
+  </si>
+  <si>
+    <t>PIMTest.java</t>
   </si>
   <si>
     <t>Aryan Chaudhary</t>
   </si>
   <si>
-    <t>cart-testing</t>
-  </si>
-  <si>
-    <t>TC_CHK_01</t>
-  </si>
-  <si>
-    <t>Checkout</t>
-  </si>
-  <si>
-    <t>Verify checkout validation when Postal Code is omitted</t>
-  </si>
-  <si>
-    <t>First: John / Last: Doe / Zip: [Empty]</t>
+    <t>pim-testing</t>
+  </si>
+  <si>
+    <t>TC_MYINFO_01</t>
+  </si>
+  <si>
+    <t>My Info</t>
+  </si>
+  <si>
+    <t>Verify Personal Details section is displayed in My Info module</t>
+  </si>
+  <si>
+    <t>Authenticated session</t>
   </si>
   <si>
     <t>DEF-005</t>
   </si>
   <si>
-    <t>Test hung waiting for order confirmation page; user was blocked on step 1.</t>
-  </si>
-  <si>
-    <t>Test failed to assert mandatory field error 'Error: Postal Code is required'. Updated test flow to assert validation message.</t>
-  </si>
-  <si>
-    <t>CheckoutTest.java</t>
+    <t>AssertionError: Form inputs not yet populated when assertion executed.</t>
+  </si>
+  <si>
+    <t>Employee details fetch via REST API on page load. Added wait for Personal Details header visibility.</t>
+  </si>
+  <si>
+    <t>MyInfoTest.java</t>
   </si>
   <si>
     <t>Jyoti Gupta</t>
   </si>
   <si>
-    <t>checkout-testing</t>
-  </si>
-  <si>
-    <t>TC_CHK_02</t>
-  </si>
-  <si>
-    <t>Verify successful end-to-end order placement</t>
-  </si>
-  <si>
-    <t>John / Doe / 12345</t>
-  </si>
-  <si>
-    <t>N/A - Clean checkout flow</t>
-  </si>
-  <si>
-    <t>Order placed and 'THANK YOU FOR YOUR ORDER' banner verified</t>
-  </si>
-  <si>
-    <t>CheckoutCompleteTest.java</t>
+    <t>myinfo-testing</t>
   </si>
 </sst>
 </file>
@@ -319,15 +280,15 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -492,13 +453,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -866,10 +827,10 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1506,21 +1467,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr defaultColWidth="10.2857142857143" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.4285714285714" customWidth="1"/>
-    <col min="2" max="2" width="16.4285714285714" customWidth="1"/>
+    <col min="1" max="1" width="15.4285714285714" customWidth="1"/>
+    <col min="2" max="2" width="17.2857142857143" customWidth="1"/>
     <col min="3" max="3" width="35.7142857142857" style="1" customWidth="1"/>
-    <col min="4" max="4" width="35.5714285714286" customWidth="1"/>
+    <col min="4" max="4" width="33.1428571428571" customWidth="1"/>
     <col min="5" max="5" width="19.5714285714286" customWidth="1"/>
     <col min="6" max="6" width="9.71428571428571" customWidth="1"/>
     <col min="7" max="7" width="45.7142857142857" style="1" customWidth="1"/>
     <col min="8" max="8" width="50.7142857142857" style="1" customWidth="1"/>
     <col min="9" max="9" width="20.2857142857143" customWidth="1"/>
-    <col min="10" max="10" width="32.2857142857143" customWidth="1"/>
+    <col min="10" max="10" width="17.8571428571429" customWidth="1"/>
     <col min="11" max="11" width="17.4285714285714" customWidth="1"/>
-    <col min="12" max="12" width="17.2857142857143" customWidth="1"/>
+    <col min="12" max="12" width="20.4285714285714" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:12">
@@ -1561,7 +1522,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" ht="30" spans="1:12">
+    <row r="2" ht="60" spans="1:12">
       <c r="A2" s="4" t="s">
         <v>12</v>
       </c>
@@ -1586,25 +1547,25 @@
       <c r="H2" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="6" t="s">
-        <v>16</v>
+      <c r="I2" s="7" t="s">
+        <v>20</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" ht="45" spans="1:12">
       <c r="A3" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>25</v>
@@ -1612,295 +1573,257 @@
       <c r="D3" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="G3" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="I3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" ht="30" spans="1:12">
+      <c r="A4" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="I3" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J3" s="4" t="s">
+      <c r="B4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="D4" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="L3" s="4" t="s">
+      <c r="K4" s="4" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="4" ht="45" spans="1:12">
-      <c r="A4" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="I4" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>21</v>
-      </c>
       <c r="L4" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" ht="30" spans="1:12">
       <c r="A5" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" ht="30" spans="1:12">
+      <c r="A6" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="5" t="s">
+      <c r="B6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="E5" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G5" s="5" t="s">
+      <c r="E6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H6" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="I5" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="K5" s="4" t="s">
+      <c r="I6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J6" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="L5" s="4" t="s">
+      <c r="K6" s="4" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="6" spans="1:12">
-      <c r="A6" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>21</v>
-      </c>
       <c r="L6" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" ht="45" spans="1:12">
       <c r="A7" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J7" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="K7" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="L7" s="4" t="s">
         <v>53</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="K7" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="L7" s="4" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="8" ht="45" spans="1:12">
       <c r="A8" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J8" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="K8" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="L8" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="D8" s="4" t="s">
+    </row>
+    <row r="9" ht="30" spans="1:12">
+      <c r="A9" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="E8" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="4" t="s">
+      <c r="B9" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="C9" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="D9" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="I8" s="6" t="s">
+      <c r="E9" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="J8" s="4" t="s">
+      <c r="F9" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="K8" s="4" t="s">
+      <c r="G9" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="L8" s="4" t="s">
+      <c r="H9" s="5" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="9" ht="45" spans="1:12">
-      <c r="A9" s="4" t="s">
+      <c r="I9" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J9" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="K9" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="L9" s="4" t="s">
         <v>73</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="K9" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="L9" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="10" ht="30" spans="1:12">
-      <c r="A10" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="L10" s="4" t="s">
-        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>